<commit_message>
Practica obligatoria Sprint 5, unidad 2
</commit_message>
<xml_diff>
--- a/03_Data_Analysis/Sprint_05/Unidad_02_Procesado_Datos_Internos_Ficheros/02_Ejercicios_Workout/data/dataset_eventos_excel.xlsx
+++ b/03_Data_Analysis/Sprint_05/Unidad_02_Procesado_Datos_Internos_Ficheros/02_Ejercicios_Workout/data/dataset_eventos_excel.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,24 +417,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>año</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>acontecimiento</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>lugar</t>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>lugares</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -464,7 +452,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -482,7 +470,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -500,7 +488,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">
@@ -518,7 +506,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="n">
@@ -536,7 +524,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="n">
@@ -554,7 +542,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="n">
@@ -572,7 +560,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="n">
@@ -590,7 +578,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="n">
@@ -608,7 +596,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="n">
@@ -626,7 +614,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="n">
@@ -644,7 +632,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="n">
@@ -662,7 +650,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
@@ -680,7 +668,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="n">
@@ -698,7 +686,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="n">
@@ -716,7 +704,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="n">
@@ -734,7 +722,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
       <c r="B18" t="n">
@@ -752,7 +740,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
       <c r="B19" t="n">
@@ -770,7 +758,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>18</v>
       </c>
       <c r="B20" t="n">
@@ -788,7 +776,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>19</v>
       </c>
       <c r="B21" t="n">
@@ -806,7 +794,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>20</v>
       </c>
       <c r="B22" t="n">
@@ -824,7 +812,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>21</v>
       </c>
       <c r="B23" t="n">
@@ -842,7 +830,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>22</v>
       </c>
       <c r="B24" t="n">
@@ -860,7 +848,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>23</v>
       </c>
       <c r="B25" t="n">
@@ -878,7 +866,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>24</v>
       </c>
       <c r="B26" t="n">
@@ -896,7 +884,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>25</v>
       </c>
       <c r="B27" t="n">
@@ -914,7 +902,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>26</v>
       </c>
       <c r="B28" t="n">

</xml_diff>